<commit_message>
Add annotator A name in label sheet
</commit_message>
<xml_diff>
--- a/golden_set/G20_labels_annotatorA.xlsx
+++ b/golden_set/G20_labels_annotatorA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\git\ICT3113-Assignment1-P2-Group20\golden_set\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92F4AAAF-AB58-49FD-B26D-A50894B006E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C509064-A070-425E-8557-6671BA995FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Labels" sheetId="1" r:id="rId1"/>
@@ -1453,9 +1453,6 @@
     <t>Annotator A label sheet - ICT3113 P2 Group 20 (200 tickets)</t>
   </si>
   <si>
-    <t>Annotator name: ____________   Student ID: ________   Protocol version used: v1</t>
-  </si>
-  <si>
     <t>Label INDEPENDENTLY: do not discuss tickets with the other annotator, and do not use any AI tool.</t>
   </si>
   <si>
@@ -1571,6 +1568,9 @@
   </si>
   <si>
     <t>Cannot understand</t>
+  </si>
+  <si>
+    <t>Annotator name: CHENG YI ZHEN  Student ID: 2402634   Protocol version used: v1</t>
   </si>
 </sst>
 </file>
@@ -1617,16 +1617,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1974,10 +1967,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -1992,10 +1985,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -2010,10 +2003,10 @@
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>415</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -2028,10 +2021,10 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -2046,10 +2039,10 @@
         <v>15</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -2064,10 +2057,10 @@
         <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -2082,10 +2075,10 @@
         <v>19</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -2100,10 +2093,10 @@
         <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F9" s="2"/>
     </row>
@@ -2118,10 +2111,10 @@
         <v>23</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F10" s="2"/>
     </row>
@@ -2136,10 +2129,10 @@
         <v>25</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F11" s="2"/>
     </row>
@@ -2154,10 +2147,10 @@
         <v>27</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -2172,10 +2165,10 @@
         <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F13" s="2"/>
     </row>
@@ -2190,10 +2183,10 @@
         <v>31</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F14" s="2"/>
     </row>
@@ -2208,10 +2201,10 @@
         <v>33</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F15" s="2"/>
     </row>
@@ -2226,10 +2219,10 @@
         <v>35</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F16" s="2"/>
     </row>
@@ -2244,10 +2237,10 @@
         <v>37</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F17" s="2"/>
     </row>
@@ -2262,10 +2255,10 @@
         <v>39</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F18" s="2"/>
     </row>
@@ -2280,10 +2273,10 @@
         <v>41</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F19" s="2"/>
     </row>
@@ -2298,10 +2291,10 @@
         <v>43</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F20" s="2"/>
     </row>
@@ -2316,10 +2309,10 @@
         <v>45</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F21" s="2"/>
     </row>
@@ -2334,10 +2327,10 @@
         <v>47</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F22" s="2"/>
     </row>
@@ -2352,10 +2345,10 @@
         <v>49</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F23" s="2"/>
     </row>
@@ -2370,10 +2363,10 @@
         <v>51</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F24" s="2"/>
     </row>
@@ -2388,10 +2381,10 @@
         <v>53</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F25" s="2"/>
     </row>
@@ -2406,10 +2399,10 @@
         <v>55</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F26" s="2"/>
     </row>
@@ -2424,10 +2417,10 @@
         <v>57</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F27" s="2"/>
     </row>
@@ -2442,10 +2435,10 @@
         <v>59</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F28" s="2"/>
     </row>
@@ -2460,10 +2453,10 @@
         <v>61</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F29" s="2"/>
     </row>
@@ -2478,10 +2471,10 @@
         <v>63</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>415</v>
       </c>
       <c r="F30" s="2"/>
     </row>
@@ -2496,10 +2489,10 @@
         <v>65</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F31" s="2"/>
     </row>
@@ -2514,10 +2507,10 @@
         <v>67</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F32" s="2"/>
     </row>
@@ -2532,10 +2525,10 @@
         <v>69</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F33" s="2"/>
     </row>
@@ -2550,13 +2543,13 @@
         <v>71</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
@@ -2570,10 +2563,10 @@
         <v>73</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="232" x14ac:dyDescent="0.35">
@@ -2587,10 +2580,10 @@
         <v>75</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F36" s="2"/>
     </row>
@@ -2605,10 +2598,10 @@
         <v>77</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F37" s="2"/>
     </row>
@@ -2623,10 +2616,10 @@
         <v>79</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F38" s="2"/>
     </row>
@@ -2641,10 +2634,10 @@
         <v>81</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F39" s="2"/>
     </row>
@@ -2659,10 +2652,10 @@
         <v>83</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F40" s="2"/>
     </row>
@@ -2677,10 +2670,10 @@
         <v>85</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F41" s="2"/>
     </row>
@@ -2695,10 +2688,10 @@
         <v>87</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F42" s="2"/>
     </row>
@@ -2713,10 +2706,10 @@
         <v>89</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F43" s="2"/>
     </row>
@@ -2731,10 +2724,10 @@
         <v>91</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F44" s="2"/>
     </row>
@@ -2749,10 +2742,10 @@
         <v>93</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F45" s="2"/>
     </row>
@@ -2767,10 +2760,10 @@
         <v>95</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F46" s="2"/>
     </row>
@@ -2785,10 +2778,10 @@
         <v>97</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F47" s="2"/>
     </row>
@@ -2803,10 +2796,10 @@
         <v>99</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F48" s="2"/>
     </row>
@@ -2821,10 +2814,10 @@
         <v>101</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="145" x14ac:dyDescent="0.35">
@@ -2838,13 +2831,13 @@
         <v>103</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E50" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="232" x14ac:dyDescent="0.35">
@@ -2858,10 +2851,10 @@
         <v>105</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F51" s="2"/>
     </row>
@@ -2876,10 +2869,10 @@
         <v>107</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F52" s="2"/>
     </row>
@@ -2894,10 +2887,10 @@
         <v>109</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F53" s="2"/>
     </row>
@@ -2912,10 +2905,10 @@
         <v>111</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F54" s="2"/>
     </row>
@@ -2930,10 +2923,10 @@
         <v>113</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F55" s="2"/>
     </row>
@@ -2948,10 +2941,10 @@
         <v>115</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F56" s="2"/>
     </row>
@@ -2966,10 +2959,10 @@
         <v>117</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F57" s="2"/>
     </row>
@@ -2984,10 +2977,10 @@
         <v>119</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F58" s="2"/>
     </row>
@@ -3002,10 +2995,10 @@
         <v>121</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F59" s="2"/>
     </row>
@@ -3020,10 +3013,10 @@
         <v>123</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F60" s="2"/>
     </row>
@@ -3038,10 +3031,10 @@
         <v>125</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F61" s="2"/>
     </row>
@@ -3056,10 +3049,10 @@
         <v>127</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F62" s="2"/>
     </row>
@@ -3074,10 +3067,10 @@
         <v>129</v>
       </c>
       <c r="D63" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>415</v>
       </c>
       <c r="F63" s="2"/>
     </row>
@@ -3092,10 +3085,10 @@
         <v>131</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F64" s="2"/>
     </row>
@@ -3110,10 +3103,10 @@
         <v>133</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F65" s="2"/>
     </row>
@@ -3128,10 +3121,10 @@
         <v>135</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F66" s="2"/>
     </row>
@@ -3146,10 +3139,10 @@
         <v>137</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F67" s="2"/>
     </row>
@@ -3164,10 +3157,10 @@
         <v>139</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F68" s="2"/>
     </row>
@@ -3182,10 +3175,10 @@
         <v>141</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F69" s="2"/>
     </row>
@@ -3200,10 +3193,10 @@
         <v>143</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F70" s="2"/>
     </row>
@@ -3218,10 +3211,10 @@
         <v>145</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F71" s="2"/>
     </row>
@@ -3236,10 +3229,10 @@
         <v>147</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F72" s="2"/>
     </row>
@@ -3254,10 +3247,10 @@
         <v>149</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F73" s="2"/>
     </row>
@@ -3272,10 +3265,10 @@
         <v>151</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F74" s="2"/>
     </row>
@@ -3290,10 +3283,10 @@
         <v>153</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F75" s="2"/>
     </row>
@@ -3308,10 +3301,10 @@
         <v>155</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F76" s="2"/>
     </row>
@@ -3326,10 +3319,10 @@
         <v>157</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="232" x14ac:dyDescent="0.35">
@@ -3343,10 +3336,10 @@
         <v>159</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F78" s="2"/>
     </row>
@@ -3361,10 +3354,10 @@
         <v>161</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F79" s="2"/>
     </row>
@@ -3379,10 +3372,10 @@
         <v>163</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F80" s="2"/>
     </row>
@@ -3397,10 +3390,10 @@
         <v>165</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F81" s="2"/>
     </row>
@@ -3415,10 +3408,10 @@
         <v>167</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F82" s="2"/>
     </row>
@@ -3433,10 +3426,10 @@
         <v>169</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F83" s="2"/>
     </row>
@@ -3451,13 +3444,13 @@
         <v>171</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
@@ -3471,13 +3464,13 @@
         <v>173</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="203" x14ac:dyDescent="0.35">
@@ -3491,10 +3484,10 @@
         <v>175</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F86" s="2"/>
     </row>
@@ -3509,10 +3502,10 @@
         <v>177</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F87" s="2"/>
     </row>
@@ -3527,13 +3520,13 @@
         <v>179</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="261" x14ac:dyDescent="0.35">
@@ -3547,10 +3540,10 @@
         <v>181</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F89" s="2"/>
     </row>
@@ -3565,13 +3558,13 @@
         <v>183</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="58" x14ac:dyDescent="0.35">
@@ -3585,10 +3578,10 @@
         <v>185</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F91" s="2"/>
     </row>
@@ -3603,10 +3596,10 @@
         <v>187</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F92" s="2"/>
     </row>
@@ -3621,10 +3614,10 @@
         <v>189</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F93" s="2"/>
     </row>
@@ -3639,10 +3632,10 @@
         <v>191</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F94" s="2"/>
     </row>
@@ -3657,10 +3650,10 @@
         <v>193</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F95" s="2"/>
     </row>
@@ -3675,10 +3668,10 @@
         <v>195</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F96" s="2"/>
     </row>
@@ -3693,10 +3686,10 @@
         <v>197</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F97" s="2"/>
     </row>
@@ -3711,13 +3704,13 @@
         <v>199</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="58" x14ac:dyDescent="0.35">
@@ -3731,10 +3724,10 @@
         <v>201</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F99" s="2"/>
     </row>
@@ -3749,10 +3742,10 @@
         <v>203</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F100" s="2"/>
     </row>
@@ -3767,10 +3760,10 @@
         <v>205</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F101" s="2"/>
     </row>
@@ -3784,13 +3777,13 @@
       <c r="C102" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="D102" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E102" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F102" s="4"/>
+      <c r="D102" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F102" s="2"/>
     </row>
     <row r="103" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
@@ -3802,14 +3795,14 @@
       <c r="C103" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="D103" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="E103" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="F103" s="4" t="s">
-        <v>443</v>
+      <c r="D103" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
@@ -3822,14 +3815,14 @@
       <c r="C104" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D104" s="4" t="s">
+      <c r="D104" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E104" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F104" s="4" t="s">
-        <v>432</v>
+      <c r="F104" s="2" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
@@ -3842,14 +3835,14 @@
       <c r="C105" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D105" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="E105" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="F105" s="4" t="s">
-        <v>431</v>
+      <c r="D105" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="145" x14ac:dyDescent="0.35">
@@ -3862,13 +3855,13 @@
       <c r="C106" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D106" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E106" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F106" s="4"/>
+      <c r="D106" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F106" s="2"/>
     </row>
     <row r="107" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
@@ -3880,13 +3873,13 @@
       <c r="C107" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D107" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E107" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F107" s="4"/>
+      <c r="D107" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F107" s="2"/>
     </row>
     <row r="108" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
@@ -3898,13 +3891,13 @@
       <c r="C108" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D108" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E108" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F108" s="4"/>
+      <c r="D108" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F108" s="2"/>
     </row>
     <row r="109" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
@@ -3916,13 +3909,13 @@
       <c r="C109" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D109" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E109" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F109" s="4"/>
+      <c r="D109" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F109" s="2"/>
     </row>
     <row r="110" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
@@ -3934,13 +3927,13 @@
       <c r="C110" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D110" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E110" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F110" s="4"/>
+      <c r="D110" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F110" s="2"/>
     </row>
     <row r="111" spans="1:6" ht="261" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
@@ -3952,13 +3945,13 @@
       <c r="C111" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="D111" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E111" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F111" s="4"/>
+      <c r="D111" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F111" s="2"/>
     </row>
     <row r="112" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
@@ -3970,13 +3963,13 @@
       <c r="C112" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="D112" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E112" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F112" s="4"/>
+      <c r="D112" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F112" s="2"/>
     </row>
     <row r="113" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
@@ -3988,13 +3981,13 @@
       <c r="C113" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D113" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E113" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F113" s="4"/>
+      <c r="D113" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F113" s="2"/>
     </row>
     <row r="114" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
@@ -4006,13 +3999,13 @@
       <c r="C114" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="D114" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E114" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F114" s="4"/>
+      <c r="D114" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F114" s="2"/>
     </row>
     <row r="115" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
@@ -4024,13 +4017,13 @@
       <c r="C115" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="D115" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E115" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F115" s="4"/>
+      <c r="D115" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F115" s="2"/>
     </row>
     <row r="116" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
@@ -4042,13 +4035,13 @@
       <c r="C116" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="D116" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="E116" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F116" s="4"/>
+      <c r="D116" t="s">
+        <v>421</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F116" s="2"/>
     </row>
     <row r="117" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
@@ -4060,14 +4053,14 @@
       <c r="C117" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D117" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E117" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F117" s="4" t="s">
-        <v>433</v>
+      <c r="D117" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
@@ -4080,13 +4073,13 @@
       <c r="C118" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="D118" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E118" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F118" s="4"/>
+      <c r="D118" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F118" s="2"/>
     </row>
     <row r="119" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
@@ -4098,14 +4091,14 @@
       <c r="C119" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D119" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="E119" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="F119" s="4" t="s">
-        <v>434</v>
+      <c r="D119" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="58" x14ac:dyDescent="0.35">
@@ -4118,14 +4111,14 @@
       <c r="C120" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D120" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E120" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F120" s="4" t="s">
-        <v>435</v>
+      <c r="D120" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
@@ -4138,13 +4131,13 @@
       <c r="C121" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="D121" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E121" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F121" s="4"/>
+      <c r="D121" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F121" s="2"/>
     </row>
     <row r="122" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
@@ -4156,13 +4149,13 @@
       <c r="C122" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D122" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="E122" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F122" s="4"/>
+      <c r="D122" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F122" s="2"/>
     </row>
     <row r="123" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
@@ -4174,13 +4167,13 @@
       <c r="C123" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D123" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E123" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F123" s="4"/>
+      <c r="D123" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F123" s="2"/>
     </row>
     <row r="124" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
@@ -4192,13 +4185,13 @@
       <c r="C124" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="D124" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E124" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F124" s="4"/>
+      <c r="D124" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F124" s="2"/>
     </row>
     <row r="125" spans="1:6" ht="116" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
@@ -4210,13 +4203,13 @@
       <c r="C125" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D125" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E125" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F125" s="4"/>
+      <c r="D125" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F125" s="2"/>
     </row>
     <row r="126" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
@@ -4228,13 +4221,13 @@
       <c r="C126" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="D126" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E126" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F126" s="4"/>
+      <c r="D126" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F126" s="2"/>
     </row>
     <row r="127" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
@@ -4246,13 +4239,13 @@
       <c r="C127" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="D127" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E127" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F127" s="4"/>
+      <c r="D127" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F127" s="2"/>
     </row>
     <row r="128" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
@@ -4264,13 +4257,13 @@
       <c r="C128" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D128" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E128" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F128" s="4"/>
+      <c r="D128" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F128" s="2"/>
     </row>
     <row r="129" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
@@ -4282,13 +4275,13 @@
       <c r="C129" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D129" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E129" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F129" s="4"/>
+      <c r="D129" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F129" s="2"/>
     </row>
     <row r="130" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
@@ -4300,13 +4293,13 @@
       <c r="C130" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D130" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="E130" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F130" s="4"/>
+      <c r="D130" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F130" s="2"/>
     </row>
     <row r="131" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
@@ -4318,13 +4311,13 @@
       <c r="C131" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="D131" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E131" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F131" s="4"/>
+      <c r="D131" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F131" s="2"/>
     </row>
     <row r="132" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
@@ -4336,14 +4329,14 @@
       <c r="C132" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="D132" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E132" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F132" s="4" t="s">
-        <v>436</v>
+      <c r="D132" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="87" x14ac:dyDescent="0.35">
@@ -4356,13 +4349,13 @@
       <c r="C133" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D133" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E133" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F133" s="4"/>
+      <c r="D133" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F133" s="2"/>
     </row>
     <row r="134" spans="1:6" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
@@ -4374,13 +4367,13 @@
       <c r="C134" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="D134" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E134" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F134" s="4"/>
+      <c r="D134" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F134" s="2"/>
     </row>
     <row r="135" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
@@ -4392,13 +4385,13 @@
       <c r="C135" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D135" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E135" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F135" s="4"/>
+      <c r="D135" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F135" s="2"/>
     </row>
     <row r="136" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
@@ -4410,13 +4403,13 @@
       <c r="C136" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D136" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E136" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F136" s="4"/>
+      <c r="D136" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F136" s="2"/>
     </row>
     <row r="137" spans="1:6" ht="348" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
@@ -4428,13 +4421,13 @@
       <c r="C137" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D137" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E137" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F137" s="4"/>
+      <c r="D137" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F137" s="2"/>
     </row>
     <row r="138" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
@@ -4446,14 +4439,14 @@
       <c r="C138" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="D138" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E138" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F138" s="4" t="s">
-        <v>437</v>
+      <c r="D138" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="116" x14ac:dyDescent="0.35">
@@ -4466,13 +4459,13 @@
       <c r="C139" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D139" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="E139" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F139" s="4"/>
+      <c r="D139" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F139" s="2"/>
     </row>
     <row r="140" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
@@ -4484,13 +4477,13 @@
       <c r="C140" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D140" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E140" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F140" s="4"/>
+      <c r="D140" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F140" s="2"/>
     </row>
     <row r="141" spans="1:6" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
@@ -4502,14 +4495,14 @@
       <c r="C141" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="D141" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E141" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F141" s="4" t="s">
-        <v>438</v>
+      <c r="D141" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>437</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="116" x14ac:dyDescent="0.35">
@@ -4522,13 +4515,13 @@
       <c r="C142" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D142" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E142" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F142" s="4"/>
+      <c r="D142" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F142" s="2"/>
     </row>
     <row r="143" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
@@ -4540,13 +4533,13 @@
       <c r="C143" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D143" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E143" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F143" s="4"/>
+      <c r="D143" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F143" s="2"/>
     </row>
     <row r="144" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
@@ -4558,13 +4551,13 @@
       <c r="C144" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="D144" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="E144" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F144" s="4"/>
+      <c r="D144" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F144" s="2"/>
     </row>
     <row r="145" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
@@ -4576,13 +4569,13 @@
       <c r="C145" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="D145" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="E145" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F145" s="4"/>
+      <c r="D145" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F145" s="2"/>
     </row>
     <row r="146" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
@@ -4594,14 +4587,14 @@
       <c r="C146" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="D146" s="4" t="s">
+      <c r="D146" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E146" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E146" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F146" s="4" t="s">
-        <v>439</v>
+      <c r="F146" s="2" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="147" spans="1:6" ht="87" x14ac:dyDescent="0.35">
@@ -4614,14 +4607,14 @@
       <c r="C147" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D147" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E147" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="F147" s="4" t="s">
-        <v>440</v>
+      <c r="D147" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="148" spans="1:6" ht="203" x14ac:dyDescent="0.35">
@@ -4634,14 +4627,14 @@
       <c r="C148" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D148" s="4" t="s">
+      <c r="D148" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E148" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E148" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F148" s="4" t="s">
-        <v>441</v>
+      <c r="F148" s="2" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="149" spans="1:6" ht="203" x14ac:dyDescent="0.35">
@@ -4654,13 +4647,13 @@
       <c r="C149" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="D149" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="E149" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F149" s="4"/>
+      <c r="D149" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F149" s="2"/>
     </row>
     <row r="150" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
@@ -4672,13 +4665,13 @@
       <c r="C150" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D150" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="E150" s="4" t="s">
-        <v>416</v>
-      </c>
-      <c r="F150" s="4"/>
+      <c r="D150" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F150" s="2"/>
     </row>
     <row r="151" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
@@ -4690,14 +4683,14 @@
       <c r="C151" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="D151" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="E151" s="4" t="s">
+      <c r="D151" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="F151" s="4" t="s">
-        <v>442</v>
+      <c r="E151" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="152" spans="1:6" ht="217.5" x14ac:dyDescent="0.35">
@@ -4710,13 +4703,13 @@
       <c r="C152" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="D152" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E152" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F152" s="5"/>
+      <c r="D152" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F152" s="2"/>
     </row>
     <row r="153" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
@@ -4728,12 +4721,12 @@
       <c r="C153" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D153" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="E153" s="5"/>
-      <c r="F153" s="5" t="s">
-        <v>444</v>
+      <c r="D153" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E153" s="2"/>
+      <c r="F153" s="2" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="154" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
@@ -4746,13 +4739,13 @@
       <c r="C154" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="D154" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E154" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F154" s="5"/>
+      <c r="D154" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F154" s="2"/>
     </row>
     <row r="155" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
@@ -4764,13 +4757,13 @@
       <c r="C155" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="D155" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E155" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F155" s="5"/>
+      <c r="D155" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F155" s="2"/>
     </row>
     <row r="156" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
@@ -4782,13 +4775,13 @@
       <c r="C156" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D156" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="E156" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F156" s="5"/>
+      <c r="D156" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F156" s="2"/>
     </row>
     <row r="157" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
@@ -4800,13 +4793,13 @@
       <c r="C157" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="D157" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E157" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F157" s="5"/>
+      <c r="D157" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F157" s="2"/>
     </row>
     <row r="158" spans="1:6" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
@@ -4818,13 +4811,13 @@
       <c r="C158" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="D158" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E158" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F158" s="5"/>
+      <c r="D158" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F158" s="2"/>
     </row>
     <row r="159" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
@@ -4836,13 +4829,13 @@
       <c r="C159" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D159" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E159" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F159" s="5"/>
+      <c r="D159" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F159" s="2"/>
     </row>
     <row r="160" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
@@ -4854,13 +4847,13 @@
       <c r="C160" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="D160" s="5" t="s">
+      <c r="D160" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E160" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E160" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F160" s="5"/>
+      <c r="F160" s="2"/>
     </row>
     <row r="161" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
@@ -4872,13 +4865,13 @@
       <c r="C161" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="D161" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E161" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F161" s="5"/>
+      <c r="D161" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F161" s="2"/>
     </row>
     <row r="162" spans="1:6" ht="406" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
@@ -4890,13 +4883,13 @@
       <c r="C162" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="D162" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="E162" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F162" s="5"/>
+      <c r="D162" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F162" s="2"/>
     </row>
     <row r="163" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
@@ -4908,14 +4901,14 @@
       <c r="C163" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="D163" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="E163" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F163" s="5" t="s">
-        <v>445</v>
+      <c r="D163" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="164" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
@@ -4928,13 +4921,13 @@
       <c r="C164" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="D164" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="E164" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F164" s="5"/>
+      <c r="D164" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F164" s="2"/>
     </row>
     <row r="165" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
@@ -4946,13 +4939,13 @@
       <c r="C165" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D165" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E165" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F165" s="5"/>
+      <c r="D165" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F165" s="2"/>
     </row>
     <row r="166" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
@@ -4964,13 +4957,13 @@
       <c r="C166" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D166" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E166" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F166" s="5"/>
+      <c r="D166" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F166" s="2"/>
     </row>
     <row r="167" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
@@ -4982,13 +4975,13 @@
       <c r="C167" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="D167" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E167" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F167" s="5"/>
+      <c r="D167" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F167" s="2"/>
     </row>
     <row r="168" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
@@ -5000,13 +4993,13 @@
       <c r="C168" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="D168" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E168" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F168" s="5"/>
+      <c r="D168" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F168" s="2"/>
     </row>
     <row r="169" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
@@ -5018,13 +5011,13 @@
       <c r="C169" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="D169" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="E169" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F169" s="5"/>
+      <c r="D169" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F169" s="2"/>
     </row>
     <row r="170" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
@@ -5036,13 +5029,13 @@
       <c r="C170" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="D170" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E170" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F170" s="5"/>
+      <c r="D170" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F170" s="2"/>
     </row>
     <row r="171" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
@@ -5054,13 +5047,13 @@
       <c r="C171" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="D171" s="5" t="s">
+      <c r="D171" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E171" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E171" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F171" s="5"/>
+      <c r="F171" s="2"/>
     </row>
     <row r="172" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
@@ -5072,13 +5065,13 @@
       <c r="C172" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D172" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E172" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F172" s="5"/>
+      <c r="D172" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F172" s="2"/>
     </row>
     <row r="173" spans="1:6" ht="174" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
@@ -5090,13 +5083,13 @@
       <c r="C173" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="D173" s="5" t="s">
+      <c r="D173" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E173" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E173" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F173" s="5"/>
+      <c r="F173" s="2"/>
     </row>
     <row r="174" spans="1:6" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
@@ -5108,13 +5101,13 @@
       <c r="C174" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="D174" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="E174" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F174" s="5"/>
+      <c r="D174" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F174" s="2"/>
     </row>
     <row r="175" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
@@ -5126,13 +5119,13 @@
       <c r="C175" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="D175" s="5" t="s">
+      <c r="D175" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E175" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E175" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F175" s="5"/>
+      <c r="F175" s="2"/>
     </row>
     <row r="176" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
@@ -5144,13 +5137,13 @@
       <c r="C176" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="D176" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="E176" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F176" s="5"/>
+      <c r="D176" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F176" s="2"/>
     </row>
     <row r="177" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
@@ -5162,13 +5155,13 @@
       <c r="C177" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="D177" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E177" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F177" s="5"/>
+      <c r="D177" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E177" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F177" s="2"/>
     </row>
     <row r="178" spans="1:6" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
@@ -5180,13 +5173,13 @@
       <c r="C178" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D178" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E178" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F178" s="5"/>
+      <c r="D178" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F178" s="2"/>
     </row>
     <row r="179" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
@@ -5198,13 +5191,13 @@
       <c r="C179" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="D179" s="5" t="s">
+      <c r="D179" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E179" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E179" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F179" s="5"/>
+      <c r="F179" s="2"/>
     </row>
     <row r="180" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
@@ -5216,13 +5209,13 @@
       <c r="C180" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="D180" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="E180" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F180" s="5"/>
+      <c r="D180" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F180" s="2"/>
     </row>
     <row r="181" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
@@ -5234,13 +5227,13 @@
       <c r="C181" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D181" s="5" t="s">
+      <c r="D181" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E181" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E181" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F181" s="5"/>
+      <c r="F181" s="2"/>
     </row>
     <row r="182" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
@@ -5252,13 +5245,13 @@
       <c r="C182" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="D182" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="E182" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F182" s="5"/>
+      <c r="D182" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E182" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F182" s="2"/>
     </row>
     <row r="183" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
@@ -5270,13 +5263,13 @@
       <c r="C183" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="D183" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E183" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F183" s="5"/>
+      <c r="D183" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E183" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F183" s="2"/>
     </row>
     <row r="184" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
@@ -5288,13 +5281,13 @@
       <c r="C184" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="D184" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="E184" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F184" s="5"/>
+      <c r="D184" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E184" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F184" s="2"/>
     </row>
     <row r="185" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
@@ -5306,13 +5299,13 @@
       <c r="C185" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="D185" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="E185" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F185" s="5"/>
+      <c r="D185" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E185" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F185" s="2"/>
     </row>
     <row r="186" spans="1:6" ht="145" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
@@ -5324,13 +5317,13 @@
       <c r="C186" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="D186" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E186" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F186" s="5"/>
+      <c r="D186" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E186" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F186" s="2"/>
     </row>
     <row r="187" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
@@ -5342,13 +5335,13 @@
       <c r="C187" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="D187" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E187" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F187" s="5"/>
+      <c r="D187" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E187" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F187" s="2"/>
     </row>
     <row r="188" spans="1:6" ht="203" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
@@ -5360,13 +5353,13 @@
       <c r="C188" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="D188" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E188" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F188" s="5"/>
+      <c r="D188" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F188" s="2"/>
     </row>
     <row r="189" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
@@ -5378,13 +5371,13 @@
       <c r="C189" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="D189" s="5" t="s">
+      <c r="D189" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E189" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E189" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F189" s="5"/>
+      <c r="F189" s="2"/>
     </row>
     <row r="190" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
@@ -5396,13 +5389,13 @@
       <c r="C190" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="D190" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E190" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F190" s="5"/>
+      <c r="D190" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E190" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F190" s="2"/>
     </row>
     <row r="191" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
@@ -5414,13 +5407,13 @@
       <c r="C191" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="D191" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="E191" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F191" s="5"/>
+      <c r="D191" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F191" s="2"/>
     </row>
     <row r="192" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
@@ -5432,14 +5425,14 @@
       <c r="C192" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="D192" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="E192" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F192" s="5" t="s">
-        <v>445</v>
+      <c r="D192" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E192" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F192" s="2" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="193" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
@@ -5452,13 +5445,13 @@
       <c r="C193" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D193" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E193" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F193" s="5"/>
+      <c r="D193" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E193" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F193" s="2"/>
     </row>
     <row r="194" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
@@ -5470,13 +5463,13 @@
       <c r="C194" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="D194" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E194" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F194" s="5"/>
+      <c r="D194" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F194" s="2"/>
     </row>
     <row r="195" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
@@ -5488,13 +5481,13 @@
       <c r="C195" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="D195" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="E195" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F195" s="5"/>
+      <c r="D195" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E195" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F195" s="2"/>
     </row>
     <row r="196" spans="1:6" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
@@ -5506,13 +5499,13 @@
       <c r="C196" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="D196" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E196" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F196" s="5"/>
+      <c r="D196" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E196" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F196" s="2"/>
     </row>
     <row r="197" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
@@ -5524,13 +5517,13 @@
       <c r="C197" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="D197" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E197" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F197" s="5"/>
+      <c r="D197" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E197" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F197" s="2"/>
     </row>
     <row r="198" spans="1:6" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
@@ -5542,13 +5535,13 @@
       <c r="C198" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="D198" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="E198" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F198" s="5"/>
+      <c r="D198" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E198" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F198" s="2"/>
     </row>
     <row r="199" spans="1:6" ht="319" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
@@ -5560,13 +5553,13 @@
       <c r="C199" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="D199" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E199" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="F199" s="5"/>
+      <c r="D199" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E199" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F199" s="2"/>
     </row>
     <row r="200" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
@@ -5578,14 +5571,14 @@
       <c r="C200" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="D200" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="E200" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="F200" s="5" t="s">
-        <v>446</v>
+      <c r="D200" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E200" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F200" s="2" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="201" spans="1:6" ht="203" x14ac:dyDescent="0.35">
@@ -5598,13 +5591,13 @@
       <c r="C201" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="D201" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="E201" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="F201" s="5"/>
+      <c r="D201" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E201" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F201" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -5634,32 +5627,32 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>407</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>